<commit_message>
Ön adım (Ö1–Ö2): YEKDEM/PPA'da batarya tutarlılığı ve nihai baz vaka
- Ö1: YEK Yönetmeliği'ne göre depolanıp verilen santral enerjisi de YEKDEM fiyatından ödenir → YEKDEM'e özgü
  dispatch (deşarj sözleşmeli fiyattan, arbitraj yok); YEKDEM'de kesinti kaybı ve batarya kurtarması yeniden
  tanımlandı; PPA finansal fark sözleşmesi (batarya tüccar dispatch'i); YEKDEM altında en iyi batarya 30 MW / 60 MWh
- Ö2: config.yaml → nihai_baz_vaka (inşaata hazır, COD 2030, RES 58,8 + 30/60, nominal YEKDEM → tüccar);
  src/07_baz_vaka.py; rapor, docs/05, docs/07, README'ler ve dashboard Özet bu kaynaktan
- Sonuç: baz vakada E[NPV] −11,4 M$, P(NPV>0) %13 → yatırım önerilmez (tüccar alternatif +0,8 M$)
- Test: YEKDEM modunda arbitraj yapılmadığı

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/07/risk_kaydi.xlsx
+++ b/outputs/07/risk_kaydi.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Risk kaydı" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk kaydı" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -784,12 +784,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>E[NPV] −2,1 M$ (öneri), −3,0 M$ (yalnız RES)</t>
+          <t>E[NPV] −2 ile −3 M$; YEKDEM'de kesilen enerjiye YEK farkı ödenmiyor</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Evet — Aşama 7 §1</t>
+          <t>Evet — Aşama 7 §1, Ö1</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -849,12 +849,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>YEKDEM'li öneri E[NPV] 5,5 (endeksli) vs 0,8 M$ (nominal)</t>
+          <t>Nihai tasarım, COD 2030: E[NPV] −3,2 (endeksli) vs −11,4 M$ (nominal)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Evet — Aşama 7 §2</t>
+          <t>Evet — Aşama 7 §2, Ö1</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>COD P50 Oca 2032 (+47 ay); E[NPV] 2,4 → −1,5 M$</t>
+          <t>COD P50 Oca 2032 (+48 ay); inşaata hazırda bile 2 yıl kayma tüccar E[NPV]'yi 4,3 → 0,8 M$ indiriyor</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Tutarlılık düzeltmeleri: YEKDEM yıllık opsiyonu, ortak batarya sürücüsü, inşaata hazır takvim
- YEKDEM: YEK Yönetmeliği md. 4/2, 5/1, 5/4, 8/1 → takvim yılı bazında yıllık katılım; 30 Kasım'da bilinen
  bilgiyle karar veren yıllık opsiyon dizisi (değerleyicide simülasyon × yıl bazında dispatch/φ)
- Ortak sürücü: kurulu batarya yolu → SFK fiyatı, sistem kesintisi ve öğle kanibalizasyonu (emilen öğle fazlası payı)
- Takvim: inşaata hazır projede bağlantı anlaşması tamam, finansman PPA'yı beklemez, türbin teslimi 12/18/30 ay →
  COD P50 Kasım 2029
- Düzeltilmiş baz vaka: E[NPV] +1,5 M$, P(NPV>0) %50, azami edinim primi ~1,5 M$; şelale ve tek başına etkiler;
  durum tespiti bilgi değeri (tavan ~1,0 M$)
- Rapor, docs/05, docs/07, README'ler, dashboard, risk kaydı güncellendi

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/07/risk_kaydi.xlsx
+++ b/outputs/07/risk_kaydi.xlsx
@@ -835,50 +835,50 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>7189 sayılı karardaki USD sınırları endekslenmezse reel değer 10 yılda ~%22 aşınır</t>
+          <t>7189 sayılı karardaki USD sınırları endekslenmezse reel değer 10 yılda ~%22 aşınır; yıllık opsiyon etkisini sınırlıyor</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
         <v>3</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Nihai tasarım, COD 2030: E[NPV] −3,2 (endeksli) vs −11,4 M$ (nominal)</t>
+          <t>Opsiyonlu baz vaka E[NPV] +3,1 (endeksli) vs +1,5 M$ (nominal); azami prim 3,1 vs 1,5 M$</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Evet — Aşama 7 §2, Ö1</t>
+          <t>Evet — docs/07 Güncelleme 2</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>FID öncesi hukuki görüş; nominal ise PPA'yı seç</t>
+          <t>Durum tespitinde hukuki görüş; teklif primini sonuca göre ayarla</t>
         </is>
       </c>
       <c r="K6" s="2" t="n">
         <v>3</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="N6" s="6" t="inlineStr">
-        <is>
-          <t>Yüksek</t>
-        </is>
-      </c>
-      <c r="O6" s="4" t="inlineStr">
-        <is>
-          <t>Orta</t>
+        <v>3</v>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>Orta</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
+        <is>
+          <t>Düşük</t>
         </is>
       </c>
     </row>
@@ -979,12 +979,12 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>COD P50 Oca 2032 (+48 ay); inşaata hazırda bile 2 yıl kayma tüccar E[NPV]'yi 4,3 → 0,8 M$ indiriyor</t>
+          <t>Geliştirmeden COD P50 May 2032; inşaata hazırda Kas 2029 ve 1,8 yıllık kayma baz vakayı 4,9 → 1,5 M$ indiriyor</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Evet — Aşama 7 §4</t>
+          <t>Evet — Aşama 7 §4, D3</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1160,7 +1160,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>OEM kapasite darboğazı, Avrupa OEM'lerinin mali zorlukları, navlun</t>
+          <t>OEM kapasite darboğazı (2024-25 teslim 18-36 ay), Avrupa OEM'lerinin mali zorlukları, navlun</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
@@ -1174,12 +1174,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Türbin tedariki kritiklik %98; CAPEX +%20 → NPV −21 M$</t>
+          <t>Türbin tedariki inşaata hazır projede kritik yolda (%100); CAPEX +%20 → NPV −21 M$</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Evet — takvim MC, tornado</t>
+          <t>Evet — takvim MC (D3), tornado</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">

</xml_diff>